<commit_message>
Fixed errors on L18
</commit_message>
<xml_diff>
--- a/CommonDesigns.xlsx
+++ b/CommonDesigns.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Jordi_Classes_234\DOE\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Jordi_Classes_245\DOE\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9155BB2-F8FB-4054-A7EE-4E736699DAE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E4375CF-6C62-4019-BF84-4D06AB3A9A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2B1F4CC8-6E29-4DF5-9B9B-812FEB45778E}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2B1F4CC8-6E29-4DF5-9B9B-812FEB45778E}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCTIONS" sheetId="17" r:id="rId1"/>
@@ -8036,7 +8036,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C11">
         <v>-1</v>
@@ -8071,7 +8071,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C12">
         <v>-1</v>
@@ -8106,7 +8106,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C13">
         <v>-1</v>
@@ -8141,7 +8141,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -8176,7 +8176,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -8211,7 +8211,7 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -8246,7 +8246,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -8281,7 +8281,7 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -8316,7 +8316,7 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C19">
         <v>1</v>

</xml_diff>